<commit_message>
chore: update workspace 2026-07-02 09:33:30
</commit_message>
<xml_diff>
--- a/新点e交易相关材料/项目服务器规划/产品服务器/企业监管平台资源清单.xlsx
+++ b/新点e交易相关材料/项目服务器规划/产品服务器/企业监管平台资源清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12291" activeTab="1"/>
+    <workbookView windowWidth="27951" windowHeight="12291" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="最小化清单" sheetId="1" r:id="rId1"/>
@@ -721,19 +721,13 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF018FFB"/>
-      <name val="Helvetica Neue"/>
-      <charset val="134"/>
-    </font>
-    <font>
+      <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
@@ -744,6 +738,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF018FFB"/>
+      <name val="Helvetica Neue"/>
       <charset val="134"/>
     </font>
   </fonts>

</xml_diff>